<commit_message>
feat: update meta tags for SEO and add 404 error pages
</commit_message>
<xml_diff>
--- a/E5.xlsx
+++ b/E5.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -33,10 +33,24 @@
     <t xml:space="preserve">NOM et prénom : PELOU Titouan</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre de formation : ESNA</t>
+    <t xml:space="preserve">N° candidat : 02248052561</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Centre de formation : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="18"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">ESNA de Bretagne – Bruz (35)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Option :</t>
@@ -45,10 +59,10 @@
     <t xml:space="preserve">▢ SISR</t>
   </si>
   <si>
-    <t xml:space="preserve">▢ SLAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse URL du portfolio : https://ahuman.fr</t>
+    <t xml:space="preserve">X SLAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adresse URL du portfolio : https://bts-2026.ahuman.fr/Portfolio/</t>
   </si>
   <si>
     <t xml:space="preserve">Compétences mises en œuvre
@@ -118,42 +132,73 @@
     <t xml:space="preserve">YODA (https://github.com/ahuman-su/YODA)</t>
   </si>
   <si>
+    <t xml:space="preserve">01/09/2025 au 15/04/2026</t>
+  </si>
+  <si>
     <t>X</t>
   </si>
   <si>
     <t xml:space="preserve">Gestionnaire de mdp (https://github.com/ahuman-su/mdp)</t>
   </si>
   <si>
+    <t xml:space="preserve">12/10/2025 au 20/12/2025</t>
+  </si>
+  <si>
     <t xml:space="preserve">C2 (https://github.com/ahuman-su/C2)</t>
   </si>
   <si>
+    <t xml:space="preserve">17/06/2025 au 15/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dévloppement d'outils de scan AD (https://github.com/BTS-ESNA-2024-2026/Projet-RADAR-B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/11/2025 au 20/11/2025</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
     <t>CUBEV2</t>
   </si>
   <si>
+    <t xml:space="preserve">01/09/2024 au 15/04/2026</t>
+  </si>
+  <si>
     <t>Suivie_projet</t>
   </si>
   <si>
+    <t xml:space="preserve">15/03/2025 au 15/04/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
     <t xml:space="preserve">Fiche reflexe</t>
   </si>
   <si>
+    <t xml:space="preserve">12/01/2026 au 22/02/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maintenance relance_auto_v20</t>
   </si>
   <si>
+    <t xml:space="preserve">02/09/2025 au 15/04/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Automatisation PMT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/02/2026 au 25/02/2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -686,18 +731,21 @@
     <xf fontId="6" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="6" fillId="0" borderId="24" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="24" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="25" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf fontId="6" fillId="0" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="24" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="7" fillId="0" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="7" fillId="0" borderId="25" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="5" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -705,9 +753,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="5" fillId="0" borderId="25" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="24" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="8" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1264,7 +1309,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="1" width="70.42578125"/>
-    <col customWidth="1" min="2" max="2" style="1" width="10.85546875"/>
+    <col customWidth="1" min="2" max="2" style="1" width="12.28125"/>
     <col customWidth="1" min="3" max="8" style="1" width="18.7109375"/>
     <col customWidth="1" min="9" max="43" width="11.42578125"/>
     <col min="44" max="16384" style="1" width="10.85546875"/>
@@ -1477,24 +1522,26 @@
       <c r="A9" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="29" t="s">
+        <v>26</v>
+      </c>
       <c r="C9" s="30" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H9" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1534,24 +1581,26 @@
     </row>
     <row r="10" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="29"/>
+        <v>28</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>29</v>
+      </c>
       <c r="C10" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" s="31"/>
       <c r="F10" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H10" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I10"/>
       <c r="J10"/>
@@ -1591,20 +1640,22 @@
     </row>
     <row r="11" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A11" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="29"/>
+        <v>30</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>31</v>
+      </c>
       <c r="C11" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="31"/>
       <c r="E11" s="31"/>
       <c r="F11" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G11" s="31"/>
       <c r="H11" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I11"/>
       <c r="J11"/>
@@ -1643,14 +1694,28 @@
       <c r="AQ11"/>
     </row>
     <row r="12" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A12" s="28"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
+      <c r="A12" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>27</v>
+      </c>
       <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="32"/>
+      <c r="F12" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="32" t="s">
+        <v>27</v>
+      </c>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1734,7 +1799,7 @@
     </row>
     <row r="14" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A14" s="28"/>
-      <c r="B14" s="29"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="31"/>
       <c r="D14" s="31"/>
       <c r="E14" s="31"/>
@@ -1779,7 +1844,7 @@
     </row>
     <row r="15" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A15" s="28"/>
-      <c r="B15" s="29"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
@@ -1824,7 +1889,7 @@
     </row>
     <row r="16" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A16" s="28"/>
-      <c r="B16" s="29"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
       <c r="E16" s="31"/>
@@ -1869,7 +1934,7 @@
     </row>
     <row r="17" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A17" s="28"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="31"/>
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
@@ -1914,7 +1979,7 @@
     </row>
     <row r="18" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A18" s="28"/>
-      <c r="B18" s="29"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="31"/>
       <c r="D18" s="31"/>
       <c r="E18" s="31"/>
@@ -1958,16 +2023,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" s="1" customFormat="1" ht="16.5">
-      <c r="A19" s="33" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="35"/>
+      <c r="A19" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="36"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -2006,26 +2071,28 @@
     </row>
     <row r="20" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A20" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="36" t="s">
-        <v>26</v>
+        <v>35</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>27</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H20" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I20"/>
       <c r="J20"/>
@@ -2065,26 +2132,28 @@
     </row>
     <row r="21" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A21" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="36" t="s">
-        <v>26</v>
+        <v>37</v>
+      </c>
+      <c r="B21" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>27</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I21"/>
       <c r="J21"/>
@@ -2124,7 +2193,7 @@
     </row>
     <row r="22" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="31"/>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -2169,7 +2238,7 @@
     </row>
     <row r="23" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A23" s="28"/>
-      <c r="B23" s="29"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="31"/>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -2214,7 +2283,7 @@
     </row>
     <row r="24" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A24" s="28"/>
-      <c r="B24" s="29"/>
+      <c r="B24" s="33"/>
       <c r="C24" s="31"/>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -2259,7 +2328,7 @@
     </row>
     <row r="25" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A25" s="28"/>
-      <c r="B25" s="29"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="31"/>
       <c r="D25" s="31"/>
       <c r="E25" s="31"/>
@@ -2304,7 +2373,7 @@
     </row>
     <row r="26" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A26" s="28"/>
-      <c r="B26" s="29"/>
+      <c r="B26" s="33"/>
       <c r="C26" s="31"/>
       <c r="D26" s="31"/>
       <c r="E26" s="31"/>
@@ -2348,16 +2417,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" s="1" customFormat="1" ht="16.5">
-      <c r="A27" s="33" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="35"/>
+      <c r="A27" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2396,18 +2465,20 @@
     </row>
     <row r="28" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A28" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="29"/>
+        <v>40</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>41</v>
+      </c>
       <c r="C28" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D28" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G28" s="31"/>
       <c r="H28" s="32"/>
@@ -2449,24 +2520,26 @@
     </row>
     <row r="29" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A29" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="29"/>
+        <v>42</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>43</v>
+      </c>
       <c r="C29" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D29" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E29" s="31"/>
       <c r="F29" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H29" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I29"/>
       <c r="J29"/>
@@ -2506,22 +2579,24 @@
     </row>
     <row r="30" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A30" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="29"/>
+        <v>44</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>45</v>
+      </c>
       <c r="C30" s="31"/>
       <c r="D30" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G30" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H30" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I30"/>
       <c r="J30"/>
@@ -2561,7 +2636,7 @@
     </row>
     <row r="31" s="1" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A31" s="28"/>
-      <c r="B31" s="29"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="31"/>
       <c r="D31" s="31"/>
       <c r="E31" s="31"/>

</xml_diff>